<commit_message>
Update YouTube dashboard data
</commit_message>
<xml_diff>
--- a/youtube_reports/YouTube_Comment_Insights_latest.xlsx
+++ b/youtube_reports/YouTube_Comment_Insights_latest.xlsx
@@ -1,5 +1,17 @@
 
-<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheets>
+    <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
+    <sheet name="Videos" sheetId="2" r:id="rId2"/>
+    <sheet name="Comments" sheetId="3" r:id="rId3"/>
+    <sheet name="Themes" sheetId="4" r:id="rId4"/>
+    <sheet name="Action Ideas" sheetId="5" r:id="rId5"/>
+  </sheets>
+</workbook>
+</file>
+
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.00%"/>
@@ -51,19 +63,7 @@
 </styleSheet>
 </file>
 
-<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheets>
-    <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
-    <sheet name="Videos" sheetId="2" r:id="rId2"/>
-    <sheet name="Comments" sheetId="3" r:id="rId3"/>
-    <sheet name="Themes" sheetId="4" r:id="rId4"/>
-    <sheet name="Action Ideas" sheetId="5" r:id="rId5"/>
-  </sheets>
-</workbook>
-</file>
-
-<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="6" max="6" width="45" customWidth="1"/>
@@ -177,7 +177,7 @@
         <v>Public views total</v>
       </c>
       <c r="B5" s="2">
-        <v>24697</v>
+        <v>24702</v>
       </c>
       <c r="C5" s="2">
         <v/>
@@ -518,7 +518,7 @@
         <v>聽起來不可思議但太多家庭都遇到一樣的問題 #shorts</v>
       </c>
       <c r="C21" s="2">
-        <v>1073</v>
+        <v>1074</v>
       </c>
       <c r="D21" s="2">
         <v>13</v>
@@ -622,10 +622,10 @@
         <v>51</v>
       </c>
       <c r="C26" s="2">
-        <v>18415</v>
+        <v>18419</v>
       </c>
       <c r="D26" s="2">
-        <v>361.1</v>
+        <v>361.2</v>
       </c>
       <c r="E26" s="2">
         <v/>
@@ -644,7 +644,7 @@
         <v>49</v>
       </c>
       <c r="C27" s="2">
-        <v>6282</v>
+        <v>6283</v>
       </c>
       <c r="D27" s="2">
         <v>128.2</v>
@@ -663,7 +663,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="9" max="9" width="10" customWidth="1"/>
@@ -737,7 +737,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>05/05/2026</t>
         </is>
       </c>
       <c r="D2" s="4">
@@ -774,14 +774,14 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>05/02/2026</t>
         </is>
       </c>
       <c r="D3" s="4">
         <f>HYPERLINK("https://www.youtube.com/watch?v=NxeVOWfGP-k","https://www.youtube.com/watch?v=NxeVOWfGP-k")</f>
       </c>
       <c r="E3" s="2">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="F3" s="2">
         <v>4</v>
@@ -790,7 +790,7 @@
         <v>0</v>
       </c>
       <c r="H3" s="3">
-        <v>0.0388</v>
+        <v>0.0377</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -811,7 +811,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>04/28/2026</t>
         </is>
       </c>
       <c r="D4" s="4">
@@ -848,7 +848,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>04/25/2026</t>
         </is>
       </c>
       <c r="D5" s="4">
@@ -885,14 +885,14 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>04/21/2026</t>
         </is>
       </c>
       <c r="D6" s="4">
         <f>HYPERLINK("https://www.youtube.com/watch?v=CGnUHEeHlts","https://www.youtube.com/watch?v=CGnUHEeHlts")</f>
       </c>
       <c r="E6" s="2">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F6" s="2">
         <v>1</v>
@@ -901,7 +901,7 @@
         <v>0</v>
       </c>
       <c r="H6" s="3">
-        <v>0.0154</v>
+        <v>0.0152</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -922,7 +922,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>04/18/2026</t>
         </is>
       </c>
       <c r="D7" s="4">
@@ -959,7 +959,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>04/14/2026</t>
         </is>
       </c>
       <c r="D8" s="4">
@@ -996,7 +996,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>04/11/2026</t>
         </is>
       </c>
       <c r="D9" s="4">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>04/07/2026</t>
         </is>
       </c>
       <c r="D10" s="4">
@@ -1070,7 +1070,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="D11" s="4">
@@ -1107,7 +1107,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>03/31/2026</t>
         </is>
       </c>
       <c r="D12" s="4">
@@ -1144,7 +1144,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>03/28/2026</t>
         </is>
       </c>
       <c r="D13" s="4">
@@ -1181,7 +1181,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>03/21/2026</t>
         </is>
       </c>
       <c r="D14" s="4">
@@ -1218,7 +1218,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>03/14/2026</t>
         </is>
       </c>
       <c r="D15" s="4">
@@ -1255,7 +1255,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>03/07/2026</t>
         </is>
       </c>
       <c r="D16" s="4">
@@ -1292,7 +1292,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>02/28/2026</t>
         </is>
       </c>
       <c r="D17" s="4">
@@ -1329,7 +1329,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>02/26/2026</t>
         </is>
       </c>
       <c r="D18" s="4">
@@ -1366,7 +1366,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>02/21/2026</t>
         </is>
       </c>
       <c r="D19" s="4">
@@ -1403,7 +1403,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>02/19/2026</t>
         </is>
       </c>
       <c r="D20" s="4">
@@ -1440,7 +1440,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>02/16/2026</t>
         </is>
       </c>
       <c r="D21" s="4">
@@ -1477,7 +1477,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>02/14/2026</t>
         </is>
       </c>
       <c r="D22" s="4">
@@ -1514,7 +1514,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>02/14/2026</t>
         </is>
       </c>
       <c r="D23" s="4">
@@ -1551,7 +1551,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>02/12/2026</t>
         </is>
       </c>
       <c r="D24" s="4">
@@ -1588,7 +1588,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>02/07/2026</t>
         </is>
       </c>
       <c r="D25" s="4">
@@ -1625,7 +1625,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>02/05/2026</t>
         </is>
       </c>
       <c r="D26" s="4">
@@ -1662,7 +1662,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>01/31/2026</t>
         </is>
       </c>
       <c r="D27" s="4">
@@ -1699,7 +1699,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>01/29/2026</t>
         </is>
       </c>
       <c r="D28" s="4">
@@ -1736,7 +1736,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>01/24/2026</t>
         </is>
       </c>
       <c r="D29" s="4">
@@ -1773,7 +1773,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>01/17/2026</t>
         </is>
       </c>
       <c r="D30" s="4">
@@ -1810,7 +1810,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>01/15/2026</t>
         </is>
       </c>
       <c r="D31" s="4">
@@ -1847,7 +1847,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>01/12/2026</t>
         </is>
       </c>
       <c r="D32" s="4">
@@ -1884,7 +1884,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>01/12/2026</t>
         </is>
       </c>
       <c r="D33" s="4">
@@ -1921,7 +1921,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>01/12/2026</t>
         </is>
       </c>
       <c r="D34" s="4">
@@ -1958,7 +1958,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>01/12/2026</t>
         </is>
       </c>
       <c r="D35" s="4">
@@ -1995,7 +1995,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>01/12/2026</t>
         </is>
       </c>
       <c r="D36" s="4">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>01/12/2026</t>
         </is>
       </c>
       <c r="D37" s="4">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="D38" s="4">
@@ -2106,7 +2106,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>01/08/2026</t>
         </is>
       </c>
       <c r="D39" s="4">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>01/03/2026</t>
         </is>
       </c>
       <c r="D40" s="4">
@@ -2180,7 +2180,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>01/03/2026</t>
         </is>
       </c>
       <c r="D41" s="4">
@@ -2217,7 +2217,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>12/30/2025</t>
         </is>
       </c>
       <c r="D42" s="4">
@@ -2254,7 +2254,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>12/27/2025</t>
         </is>
       </c>
       <c r="D43" s="4">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>12/23/2025</t>
         </is>
       </c>
       <c r="D44" s="4">
@@ -2328,7 +2328,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>12/20/2025</t>
         </is>
       </c>
       <c r="D45" s="4">
@@ -2365,7 +2365,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>12/18/2025</t>
         </is>
       </c>
       <c r="D46" s="4">
@@ -2402,7 +2402,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>12/13/2025</t>
         </is>
       </c>
       <c r="D47" s="4">
@@ -2439,7 +2439,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>12/11/2025</t>
         </is>
       </c>
       <c r="D48" s="4">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2025-12-06</t>
+          <t>12/06/2025</t>
         </is>
       </c>
       <c r="D49" s="4">
@@ -2513,7 +2513,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>12/02/2025</t>
         </is>
       </c>
       <c r="D50" s="4">
@@ -2550,7 +2550,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>11/29/2025</t>
         </is>
       </c>
       <c r="D51" s="4">
@@ -2587,7 +2587,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>11/29/2025</t>
         </is>
       </c>
       <c r="D52" s="4">
@@ -2624,7 +2624,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>11/29/2025</t>
         </is>
       </c>
       <c r="D53" s="4">
@@ -2661,7 +2661,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>11/29/2025</t>
         </is>
       </c>
       <c r="D54" s="4">
@@ -2698,7 +2698,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>11/27/2025</t>
         </is>
       </c>
       <c r="D55" s="4">
@@ -2735,7 +2735,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>11/25/2025</t>
         </is>
       </c>
       <c r="D56" s="4">
@@ -2772,7 +2772,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2025-11-22</t>
+          <t>11/22/2025</t>
         </is>
       </c>
       <c r="D57" s="4">
@@ -2809,7 +2809,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2025-11-20</t>
+          <t>11/20/2025</t>
         </is>
       </c>
       <c r="D58" s="4">
@@ -2846,7 +2846,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2025-11-18</t>
+          <t>11/18/2025</t>
         </is>
       </c>
       <c r="D59" s="4">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2025-11-15</t>
+          <t>11/15/2025</t>
         </is>
       </c>
       <c r="D60" s="4">
@@ -2920,7 +2920,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2025-11-11</t>
+          <t>11/11/2025</t>
         </is>
       </c>
       <c r="D61" s="4">
@@ -2957,7 +2957,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2025-11-08</t>
+          <t>11/08/2025</t>
         </is>
       </c>
       <c r="D62" s="4">
@@ -2994,7 +2994,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2025-11-06</t>
+          <t>11/06/2025</t>
         </is>
       </c>
       <c r="D63" s="4">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2025-11-05</t>
+          <t>11/05/2025</t>
         </is>
       </c>
       <c r="D64" s="4">
@@ -3068,7 +3068,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>2025-11-04</t>
+          <t>11/04/2025</t>
         </is>
       </c>
       <c r="D65" s="4">
@@ -3105,7 +3105,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2025-10-30</t>
+          <t>10/30/2025</t>
         </is>
       </c>
       <c r="D66" s="4">
@@ -3142,7 +3142,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2025-10-30</t>
+          <t>10/30/2025</t>
         </is>
       </c>
       <c r="D67" s="4">
@@ -3179,7 +3179,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2025-10-28</t>
+          <t>10/28/2025</t>
         </is>
       </c>
       <c r="D68" s="4">
@@ -3216,7 +3216,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2025-10-25</t>
+          <t>10/25/2025</t>
         </is>
       </c>
       <c r="D69" s="4">
@@ -3253,7 +3253,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2025-10-21</t>
+          <t>10/21/2025</t>
         </is>
       </c>
       <c r="D70" s="4">
@@ -3290,7 +3290,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2025-10-18</t>
+          <t>10/18/2025</t>
         </is>
       </c>
       <c r="D71" s="4">
@@ -3327,7 +3327,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>2025-10-16</t>
+          <t>10/16/2025</t>
         </is>
       </c>
       <c r="D72" s="4">
@@ -3364,7 +3364,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>2025-10-14</t>
+          <t>10/14/2025</t>
         </is>
       </c>
       <c r="D73" s="4">
@@ -3401,7 +3401,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>2025-10-11</t>
+          <t>10/11/2025</t>
         </is>
       </c>
       <c r="D74" s="4">
@@ -3438,7 +3438,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>2025-10-09</t>
+          <t>10/09/2025</t>
         </is>
       </c>
       <c r="D75" s="4">
@@ -3475,7 +3475,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2025-10-07</t>
+          <t>10/07/2025</t>
         </is>
       </c>
       <c r="D76" s="4">
@@ -3512,7 +3512,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>2025-10-05</t>
+          <t>10/05/2025</t>
         </is>
       </c>
       <c r="D77" s="4">
@@ -3549,7 +3549,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>2025-10-04</t>
+          <t>10/04/2025</t>
         </is>
       </c>
       <c r="D78" s="4">
@@ -3586,7 +3586,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2025-10-04</t>
+          <t>10/04/2025</t>
         </is>
       </c>
       <c r="D79" s="4">
@@ -3623,7 +3623,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2025-10-02</t>
+          <t>10/02/2025</t>
         </is>
       </c>
       <c r="D80" s="4">
@@ -3660,7 +3660,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>2025-10-01</t>
+          <t>10/01/2025</t>
         </is>
       </c>
       <c r="D81" s="4">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2025-09-30</t>
+          <t>09/30/2025</t>
         </is>
       </c>
       <c r="D82" s="4">
@@ -3734,7 +3734,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>2025-09-27</t>
+          <t>09/27/2025</t>
         </is>
       </c>
       <c r="D83" s="4">
@@ -3771,7 +3771,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>2025-09-27</t>
+          <t>09/27/2025</t>
         </is>
       </c>
       <c r="D84" s="4">
@@ -3808,14 +3808,14 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>2025-09-25</t>
+          <t>09/25/2025</t>
         </is>
       </c>
       <c r="D85" s="4">
         <f>HYPERLINK("https://www.youtube.com/watch?v=1Yp-hUO3SpA","https://www.youtube.com/watch?v=1Yp-hUO3SpA")</f>
       </c>
       <c r="E85" s="2">
-        <v>1073</v>
+        <v>1074</v>
       </c>
       <c r="F85" s="2">
         <v>13</v>
@@ -3845,7 +3845,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>2025-09-24</t>
+          <t>09/24/2025</t>
         </is>
       </c>
       <c r="D86" s="4">
@@ -3882,7 +3882,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>2025-09-20</t>
+          <t>09/20/2025</t>
         </is>
       </c>
       <c r="D87" s="4">
@@ -3919,7 +3919,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>2025-09-18</t>
+          <t>09/18/2025</t>
         </is>
       </c>
       <c r="D88" s="4">
@@ -3956,7 +3956,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>2025-09-17</t>
+          <t>09/17/2025</t>
         </is>
       </c>
       <c r="D89" s="4">
@@ -3993,7 +3993,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>2025-09-11</t>
+          <t>09/11/2025</t>
         </is>
       </c>
       <c r="D90" s="4">
@@ -4030,7 +4030,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>2025-09-10</t>
+          <t>09/10/2025</t>
         </is>
       </c>
       <c r="D91" s="4">
@@ -4067,7 +4067,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>2025-09-05</t>
+          <t>09/05/2025</t>
         </is>
       </c>
       <c r="D92" s="4">
@@ -4104,7 +4104,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>2025-09-04</t>
+          <t>09/04/2025</t>
         </is>
       </c>
       <c r="D93" s="4">
@@ -4141,7 +4141,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>2025-09-03</t>
+          <t>09/03/2025</t>
         </is>
       </c>
       <c r="D94" s="4">
@@ -4178,7 +4178,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>2025-09-03</t>
+          <t>09/03/2025</t>
         </is>
       </c>
       <c r="D95" s="4">
@@ -4215,7 +4215,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>2025-09-03</t>
+          <t>09/03/2025</t>
         </is>
       </c>
       <c r="D96" s="4">
@@ -4252,7 +4252,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>2025-08-29</t>
+          <t>08/29/2025</t>
         </is>
       </c>
       <c r="D97" s="4">
@@ -4289,7 +4289,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>2025-08-29</t>
+          <t>08/29/2025</t>
         </is>
       </c>
       <c r="D98" s="4">
@@ -4326,7 +4326,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>2025-08-27</t>
+          <t>08/27/2025</t>
         </is>
       </c>
       <c r="D99" s="4">
@@ -4363,7 +4363,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>2025-08-27</t>
+          <t>08/27/2025</t>
         </is>
       </c>
       <c r="D100" s="4">
@@ -4400,7 +4400,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2025-08-26</t>
+          <t>08/26/2025</t>
         </is>
       </c>
       <c r="D101" s="4">
@@ -4429,7 +4429,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="11" max="11" width="55" customWidth="1"/>
@@ -4523,7 +4523,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>02/08/2026</t>
         </is>
       </c>
       <c r="F2" s="2">
@@ -4576,7 +4576,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>02/08/2026</t>
         </is>
       </c>
       <c r="F3" s="2">
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>02/07/2026</t>
         </is>
       </c>
       <c r="F4" s="2">
@@ -4682,7 +4682,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>02/07/2026</t>
         </is>
       </c>
       <c r="F5" s="2">
@@ -4735,7 +4735,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>02/07/2026</t>
         </is>
       </c>
       <c r="F6" s="2">
@@ -4788,7 +4788,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>12/27/2025</t>
         </is>
       </c>
       <c r="F7" s="2">
@@ -4841,7 +4841,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>12/27/2025</t>
         </is>
       </c>
       <c r="F8" s="2">
@@ -4894,7 +4894,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>12/27/2025</t>
         </is>
       </c>
       <c r="F9" s="2">
@@ -4947,7 +4947,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2025-11-21</t>
+          <t>11/21/2025</t>
         </is>
       </c>
       <c r="F10" s="2">
@@ -5000,7 +5000,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2025-11-16</t>
+          <t>11/16/2025</t>
         </is>
       </c>
       <c r="F11" s="2">
@@ -5053,7 +5053,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2025-11-16</t>
+          <t>11/16/2025</t>
         </is>
       </c>
       <c r="F12" s="2">
@@ -5106,7 +5106,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2025-10-30</t>
+          <t>10/30/2025</t>
         </is>
       </c>
       <c r="F13" s="2">
@@ -5159,7 +5159,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2025-10-30</t>
+          <t>10/30/2025</t>
         </is>
       </c>
       <c r="F14" s="2">
@@ -5212,7 +5212,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2025-09-26</t>
+          <t>09/26/2025</t>
         </is>
       </c>
       <c r="F15" s="2">
@@ -5249,7 +5249,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="3" max="3" width="36" customWidth="1"/>
@@ -5292,7 +5292,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>孩子只說英文</t>
+          <t>共讀與閱讀</t>
         </is>
       </c>
       <c r="B3" s="2">
@@ -5307,7 +5307,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>共讀與閱讀</t>
+          <t>海外環境</t>
         </is>
       </c>
       <c r="B4" s="2">
@@ -5322,7 +5322,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>海外環境</t>
+          <t>孩子只說英文</t>
         </is>
       </c>
       <c r="B5" s="2">
@@ -5339,7 +5339,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="4" max="4" width="12" customWidth="1"/>

</xml_diff>